<commit_message>
fix: update debuger free doc
</commit_message>
<xml_diff>
--- a/CANoe_Replacement_Requirements.xlsx
+++ b/CANoe_Replacement_Requirements.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selection Criteria" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debugger-Free Flashing Req" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flash Acceptance KPI" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1510,4 +1512,839 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Req ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Detailed Requirement</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Rationale</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Verification Method</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Notes / Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DFR-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Line Architecture</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>EOL line shall operate without J-Link and Trace32 for production flashing and test execution.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Reduce tooling cost and simplify station hardware</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Architecture review and station inspection</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>System Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>DFR-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Flashing Transport</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>DUT firmware flashing shall be performed over CAN or LIN transport according to approved protocol.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Core replacement objective</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>End-to-end flashing test</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Firmware + Software</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>DFR-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Bootloader Entry</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>System shall support deterministic bootloader entry via EOL command sequence and power/reset control.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Reliable production automation</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Repeated entry/exit validation</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Firmware Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>DFR-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Image Integrity</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Flashing flow shall validate image integrity using CRC or stronger cryptographic integrity check before activation.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Prevent corrupted firmware deployment</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Corruption injection test</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Firmware + Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>DFR-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Security Access</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Flashing path shall enforce required security unlock mechanism before allowing memory programming.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Prevent unauthorized programming</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Security access test cases</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Cybersecurity</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>DFR-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Chunk Transfer</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Flashing implementation shall support segmented data transfer with configurable block size and timeout handling.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Large image support and robustness</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Stress flashing with max image size</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Software Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>DFR-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Retry and Resume</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>On recoverable communication failure, flasher shall retry and optionally resume transfer from last acknowledged block.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Improve station uptime</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Cable disturbance test</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Software Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>DFR-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Atomic Activation</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Firmware activation shall occur only after full successful transfer and verification.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Avoid bricked or undefined state</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Power interruption scenario tests</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Firmware Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>DFR-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Post-Flash Verify</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Station shall verify programmed version and checksum/signature immediately after flashing.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Ensure programmed image correctness</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Automated post-flash verification</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Validation Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>DFR-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Flash KPI</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Station shall log flash duration, success/failure code, retry count, and verification result per DUT.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Traceability and optimization</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>CSV/Excel report inspection</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Quality + Software</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>DFR-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Barcode Binding</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Flash and test records shall be bound to scanned 19-character barcode and derived 16-digit serial.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Unit-level traceability</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Report cross-check</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing + Software</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>DFR-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Cycle Time</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Average flash + test cycle shall stay within agreed takt-time limit for production line.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Throughput protection</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Pilot KPI measurement</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>DFR-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Recovery SOP</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Operator SOP shall define safe recovery actions for flash fail, verify fail, and communication fail cases.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Reduce line downtime</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>SOP dry run</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>DFR-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Fallback</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>System shall support controlled fallback path when flashing cannot complete (quarantine / retest station handling).</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Containment and quality control</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Pilot containment drill</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Quality Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>DFR-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Version Control</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Released station image shall lock flasher version, protocol config, and approved firmware package versions.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable production behavior</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Release audit</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Configuration Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>DFR-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Scalability</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Debugger-free flashing solution shall support rollout to multiple stations with consistent behavior.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Factory scalability</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Multi-station validation</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Measurement Window</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Pass Criteria</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Flash success rate</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>&gt;= 99.0%</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Pilot lot</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Successful programmed + verified DUTs / attempted DUTs</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Validation Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Average flash time</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>As per takt budget</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Pilot lot</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Mean flash duration within agreed limit</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing Eng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Recovery success</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>&gt;= 95%</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Fault-injection runs</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Recoverable failures resolved without manual reprogramming tools</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Software Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>False fail rate</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>&lt;= 1.0%</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Pilot lot</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Failures reproduced and confirmed as true defects</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Quality Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Traceability completeness</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Pilot lot</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Each DUT has barcode, flash result, and test result in report logs</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Quality + IT</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>